<commit_message>
[feat/ASP-2684-Module-Activity-Report] Addressed review comments
</commit_message>
<xml_diff>
--- a/api/templates/module_activity_report/en.xlsx
+++ b/api/templates/module_activity_report/en.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\ahernandez\repos\aspect\api\templates\module_activity_report\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\ahernandez\repos\aspect\api\templates\module_activity_report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EE50B2A-F1A6-4B8E-B2D1-BE4149B70713}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C105662-97A6-4017-8797-D80D4182DC06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{3EE22C30-721D-4358-A9D5-5FEF2B321F4D}"/>
   </bookViews>
@@ -85,16 +85,16 @@
     <t>Module Activity Report</t>
   </si>
   <si>
-    <t>Cities: &lt;Lgas&gt;</t>
-  </si>
-  <si>
-    <t>Provinces:  &lt;States&gt;</t>
-  </si>
-  <si>
     <t>Date Last Issue</t>
   </si>
   <si>
     <t>&lt;dateLastIssue&gt;</t>
+  </si>
+  <si>
+    <t>States/Provinces:  &lt;States&gt;</t>
+  </si>
+  <si>
+    <t>Cities/Lgas: &lt;Lgas&gt;</t>
   </si>
 </sst>
 </file>
@@ -541,13 +541,13 @@
     </row>
     <row r="3" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B3" s="4"/>
     </row>
     <row r="4" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="B4" s="4"/>
     </row>
@@ -573,7 +573,7 @@
         <v>8</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="G7" s="5" t="s">
         <v>12</v>
@@ -596,7 +596,7 @@
         <v>4</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="G8" s="2" t="s">
         <v>13</v>

</xml_diff>